<commit_message>
Update template paths in ig.ini f5f95e57033fc75d57dba400d8f7e732c9d81c11
</commit_message>
<xml_diff>
--- a/nriss-patch-2/ig/StructureDefinition-fr-accession-number-identifier-document.xlsx
+++ b/nriss-patch-2/ig/StructureDefinition-fr-accession-number-identifier-document.xlsx
@@ -10,13 +10,13 @@
     <sheet name="Elements" r:id="rId4" sheetId="2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">Elements!$A$1:$AM$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">Elements!$A$1:$AM$16</definedName>
   </definedNames>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="391" uniqueCount="160">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="605" uniqueCount="185">
   <si>
     <t>Property</t>
   </si>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-08-07T09:15:45+00:00</t>
+    <t>2026-10-01T07:42:11+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -394,15 +394,6 @@
     <t>Allows users to make use of identifiers when the identifier system is not known.</t>
   </si>
   <si>
-    <t>&lt;valueCodeableConcept xmlns="http://hl7.org/fhir"&gt;
-  &lt;coding&gt;
-    &lt;system value="http://terminology.hl7.org/CodeSystem/v2-0203"/&gt;
-    &lt;code value="ACSN"/&gt;
-    &lt;display value="Accession ID"/&gt;
-  &lt;/coding&gt;
-&lt;/valueCodeableConcept&gt;</t>
-  </si>
-  <si>
     <t>extensible</t>
   </si>
   <si>
@@ -413,6 +404,93 @@
   </si>
   <si>
     <t>CX.5</t>
+  </si>
+  <si>
+    <t>Identifier.type.id</t>
+  </si>
+  <si>
+    <t>Identifier.type.extension</t>
+  </si>
+  <si>
+    <t>Identifier.type.coding</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Coding
+</t>
+  </si>
+  <si>
+    <t>Code defined by a terminology system</t>
+  </si>
+  <si>
+    <t>A reference to a code defined by a terminology system.</t>
+  </si>
+  <si>
+    <t>Codes may be defined very casually in enumerations, or code lists, up to very formal definitions such as SNOMED CT - see the HL7 v3 Core Principles for more information.  Ordering of codings is undefined and SHALL NOT be used to infer meaning. Generally, at most only one of the coding values will be labeled as UserSelected = true.</t>
+  </si>
+  <si>
+    <t>Allows for alternative encodings within a code system, and translations to other code systems.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">value:$this}
+</t>
+  </si>
+  <si>
+    <t>CodeableConcept.coding</t>
+  </si>
+  <si>
+    <t>C*E.1-8, C*E.10-22</t>
+  </si>
+  <si>
+    <t>union(., ./translation)</t>
+  </si>
+  <si>
+    <t>Identifier.type.coding:v2-0203-coding</t>
+  </si>
+  <si>
+    <t>v2-0203-coding</t>
+  </si>
+  <si>
+    <t>&lt;valueCoding xmlns="http://hl7.org/fhir"&gt;
+  &lt;system value="http://terminology.hl7.org/CodeSystem/v2-0203"/&gt;
+  &lt;code value="ACSN"/&gt;
+&lt;/valueCoding&gt;</t>
+  </si>
+  <si>
+    <t>Identifier.type.coding:dcm</t>
+  </si>
+  <si>
+    <t>dcm</t>
+  </si>
+  <si>
+    <t>&lt;valueCoding xmlns="http://hl7.org/fhir"&gt;
+  &lt;system value="http://dicom.nema.org/resources/ontology/DCM"/&gt;
+  &lt;code value="121022"/&gt;
+  &lt;display value="Accession Number"/&gt;
+&lt;/valueCoding&gt;</t>
+  </si>
+  <si>
+    <t>Identifier.type.text</t>
+  </si>
+  <si>
+    <t>Plain text representation of the concept</t>
+  </si>
+  <si>
+    <t>A human language representation of the concept as seen/selected/uttered by the user who entered the data and/or which represents the intended meaning of the user.</t>
+  </si>
+  <si>
+    <t>Very often the text is the same as a displayName of one of the codings.</t>
+  </si>
+  <si>
+    <t>The codes from the terminologies do not always capture the correct meaning with all the nuances of the human using them, or sometimes there is no appropriate code at all. In these cases, the text is used to capture the full meaning of the source.</t>
+  </si>
+  <si>
+    <t>CodeableConcept.text</t>
+  </si>
+  <si>
+    <t>C*E.9. But note many systems use C*E.2 for this</t>
+  </si>
+  <si>
+    <t>./originalText[mediaType/code="text/plain"]/data</t>
   </si>
   <si>
     <t>Identifier.system</t>
@@ -831,12 +909,12 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AM10"/>
+  <dimension ref="A1:AM16"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="16.1640625" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="16.1640625" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="10.8515625" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="1" max="1" width="30.58984375" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="20.17578125" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="13.21484375" customWidth="true" bestFit="true" hidden="true"/>
     <col min="4" max="4" width="10.83984375" customWidth="true" bestFit="true" hidden="true"/>
     <col min="5" max="5" width="5.80859375" customWidth="true" bestFit="true"/>
     <col min="6" max="6" width="4.23828125" customWidth="true" bestFit="true"/>
@@ -848,7 +926,7 @@
     <col min="12" max="12" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="13" max="13" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="14" max="14" width="100.703125" customWidth="true" bestFit="true"/>
-    <col min="15" max="15" width="143.54296875" customWidth="true" bestFit="true"/>
+    <col min="15" max="15" width="196.6875" customWidth="true" bestFit="true"/>
     <col min="16" max="16" width="20.703125" customWidth="true" bestFit="true"/>
     <col min="17" max="17" width="20.703125" customWidth="true" bestFit="true"/>
     <col min="18" max="18" width="20.703125" customWidth="true" bestFit="true"/>
@@ -865,7 +943,7 @@
     <col min="29" max="29" width="36.0390625" customWidth="true" bestFit="true"/>
     <col min="30" max="30" width="14.7578125" customWidth="true" bestFit="true"/>
     <col min="31" max="31" width="12.359375" customWidth="true" bestFit="true" hidden="true"/>
-    <col min="32" max="32" width="15.59375" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="32" max="32" width="20.5390625" customWidth="true" bestFit="true" hidden="true"/>
     <col min="33" max="33" width="9.046875" customWidth="true" bestFit="true" hidden="true"/>
     <col min="34" max="34" width="9.46484375" customWidth="true" bestFit="true"/>
     <col min="35" max="35" width="100.703125" customWidth="true"/>
@@ -1485,28 +1563,28 @@
         <v>76</v>
       </c>
       <c r="S6" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="T6" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="U6" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="V6" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="W6" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="X6" t="s" s="2">
         <v>122</v>
       </c>
-      <c r="T6" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="U6" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="V6" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="W6" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="X6" t="s" s="2">
+      <c r="Y6" t="s" s="2">
         <v>123</v>
       </c>
-      <c r="Y6" t="s" s="2">
+      <c r="Z6" t="s" s="2">
         <v>124</v>
-      </c>
-      <c r="Z6" t="s" s="2">
-        <v>125</v>
       </c>
       <c r="AA6" t="s" s="2">
         <v>76</v>
@@ -1539,7 +1617,7 @@
         <v>83</v>
       </c>
       <c r="AK6" t="s" s="2">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="AL6" t="s" s="2">
         <v>115</v>
@@ -1548,12 +1626,12 @@
         <v>76</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" hidden="true">
       <c r="A7" t="s" s="2">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B7" t="s" s="2">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C7" s="2"/>
       <c r="D7" t="s" s="2">
@@ -1567,29 +1645,25 @@
         <v>87</v>
       </c>
       <c r="H7" t="s" s="2">
-        <v>105</v>
+        <v>76</v>
       </c>
       <c r="I7" t="s" s="2">
         <v>76</v>
       </c>
       <c r="J7" t="s" s="2">
-        <v>105</v>
+        <v>76</v>
       </c>
       <c r="K7" t="s" s="2">
-        <v>128</v>
+        <v>88</v>
       </c>
       <c r="L7" t="s" s="2">
-        <v>129</v>
+        <v>89</v>
       </c>
       <c r="M7" t="s" s="2">
-        <v>130</v>
-      </c>
-      <c r="N7" t="s" s="2">
-        <v>131</v>
-      </c>
-      <c r="O7" t="s" s="2">
-        <v>132</v>
-      </c>
+        <v>90</v>
+      </c>
+      <c r="N7" s="2"/>
+      <c r="O7" s="2"/>
       <c r="P7" t="s" s="2">
         <v>76</v>
       </c>
@@ -1601,7 +1675,7 @@
         <v>76</v>
       </c>
       <c r="T7" t="s" s="2">
-        <v>133</v>
+        <v>76</v>
       </c>
       <c r="U7" t="s" s="2">
         <v>76</v>
@@ -1637,7 +1711,7 @@
         <v>76</v>
       </c>
       <c r="AF7" t="s" s="2">
-        <v>127</v>
+        <v>91</v>
       </c>
       <c r="AG7" t="s" s="2">
         <v>77</v>
@@ -1649,56 +1723,56 @@
         <v>76</v>
       </c>
       <c r="AJ7" t="s" s="2">
-        <v>83</v>
+        <v>76</v>
       </c>
       <c r="AK7" t="s" s="2">
-        <v>134</v>
+        <v>76</v>
       </c>
       <c r="AL7" t="s" s="2">
-        <v>135</v>
+        <v>92</v>
       </c>
       <c r="AM7" t="s" s="2">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="8">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="8" hidden="true">
       <c r="A8" t="s" s="2">
-        <v>137</v>
+        <v>127</v>
       </c>
       <c r="B8" t="s" s="2">
-        <v>137</v>
+        <v>127</v>
       </c>
       <c r="C8" s="2"/>
       <c r="D8" t="s" s="2">
-        <v>76</v>
+        <v>94</v>
       </c>
       <c r="E8" s="2"/>
       <c r="F8" t="s" s="2">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="G8" t="s" s="2">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="H8" t="s" s="2">
-        <v>105</v>
+        <v>76</v>
       </c>
       <c r="I8" t="s" s="2">
         <v>76</v>
       </c>
       <c r="J8" t="s" s="2">
-        <v>105</v>
+        <v>76</v>
       </c>
       <c r="K8" t="s" s="2">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="L8" t="s" s="2">
-        <v>138</v>
+        <v>96</v>
       </c>
       <c r="M8" t="s" s="2">
-        <v>139</v>
+        <v>97</v>
       </c>
       <c r="N8" t="s" s="2">
-        <v>140</v>
+        <v>98</v>
       </c>
       <c r="O8" s="2"/>
       <c r="P8" t="s" s="2">
@@ -1712,7 +1786,7 @@
         <v>76</v>
       </c>
       <c r="T8" t="s" s="2">
-        <v>141</v>
+        <v>76</v>
       </c>
       <c r="U8" t="s" s="2">
         <v>76</v>
@@ -1736,48 +1810,48 @@
         <v>76</v>
       </c>
       <c r="AB8" t="s" s="2">
-        <v>76</v>
+        <v>99</v>
       </c>
       <c r="AC8" t="s" s="2">
-        <v>76</v>
+        <v>100</v>
       </c>
       <c r="AD8" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AE8" t="s" s="2">
-        <v>76</v>
+        <v>101</v>
       </c>
       <c r="AF8" t="s" s="2">
-        <v>137</v>
+        <v>102</v>
       </c>
       <c r="AG8" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH8" t="s" s="2">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="AI8" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AJ8" t="s" s="2">
-        <v>83</v>
+        <v>103</v>
       </c>
       <c r="AK8" t="s" s="2">
-        <v>142</v>
+        <v>76</v>
       </c>
       <c r="AL8" t="s" s="2">
-        <v>143</v>
+        <v>92</v>
       </c>
       <c r="AM8" t="s" s="2">
-        <v>144</v>
+        <v>76</v>
       </c>
     </row>
     <row r="9" hidden="true">
       <c r="A9" t="s" s="2">
-        <v>145</v>
+        <v>128</v>
       </c>
       <c r="B9" t="s" s="2">
-        <v>145</v>
+        <v>128</v>
       </c>
       <c r="C9" s="2"/>
       <c r="D9" t="s" s="2">
@@ -1785,10 +1859,10 @@
       </c>
       <c r="E9" s="2"/>
       <c r="F9" t="s" s="2">
-        <v>77</v>
+        <v>87</v>
       </c>
       <c r="G9" t="s" s="2">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="H9" t="s" s="2">
         <v>76</v>
@@ -1800,16 +1874,20 @@
         <v>105</v>
       </c>
       <c r="K9" t="s" s="2">
-        <v>146</v>
+        <v>129</v>
       </c>
       <c r="L9" t="s" s="2">
-        <v>147</v>
+        <v>130</v>
       </c>
       <c r="M9" t="s" s="2">
-        <v>148</v>
-      </c>
-      <c r="N9" s="2"/>
-      <c r="O9" s="2"/>
+        <v>131</v>
+      </c>
+      <c r="N9" t="s" s="2">
+        <v>132</v>
+      </c>
+      <c r="O9" t="s" s="2">
+        <v>133</v>
+      </c>
       <c r="P9" t="s" s="2">
         <v>76</v>
       </c>
@@ -1845,25 +1923,23 @@
         <v>76</v>
       </c>
       <c r="AB9" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AC9" t="s" s="2">
-        <v>76</v>
-      </c>
+        <v>134</v>
+      </c>
+      <c r="AC9" s="2"/>
       <c r="AD9" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AE9" t="s" s="2">
-        <v>76</v>
+        <v>101</v>
       </c>
       <c r="AF9" t="s" s="2">
-        <v>145</v>
+        <v>135</v>
       </c>
       <c r="AG9" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH9" t="s" s="2">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="AI9" t="s" s="2">
         <v>76</v>
@@ -1872,29 +1948,31 @@
         <v>83</v>
       </c>
       <c r="AK9" t="s" s="2">
-        <v>149</v>
+        <v>136</v>
       </c>
       <c r="AL9" t="s" s="2">
-        <v>150</v>
+        <v>137</v>
       </c>
       <c r="AM9" t="s" s="2">
-        <v>151</v>
+        <v>76</v>
       </c>
     </row>
     <row r="10" hidden="true">
       <c r="A10" t="s" s="2">
-        <v>152</v>
+        <v>138</v>
       </c>
       <c r="B10" t="s" s="2">
-        <v>152</v>
-      </c>
-      <c r="C10" s="2"/>
+        <v>128</v>
+      </c>
+      <c r="C10" t="s" s="2">
+        <v>139</v>
+      </c>
       <c r="D10" t="s" s="2">
         <v>76</v>
       </c>
       <c r="E10" s="2"/>
       <c r="F10" t="s" s="2">
-        <v>77</v>
+        <v>87</v>
       </c>
       <c r="G10" t="s" s="2">
         <v>87</v>
@@ -1909,18 +1987,20 @@
         <v>105</v>
       </c>
       <c r="K10" t="s" s="2">
-        <v>153</v>
+        <v>129</v>
       </c>
       <c r="L10" t="s" s="2">
-        <v>154</v>
+        <v>130</v>
       </c>
       <c r="M10" t="s" s="2">
-        <v>155</v>
+        <v>131</v>
       </c>
       <c r="N10" t="s" s="2">
-        <v>156</v>
-      </c>
-      <c r="O10" s="2"/>
+        <v>132</v>
+      </c>
+      <c r="O10" t="s" s="2">
+        <v>133</v>
+      </c>
       <c r="P10" t="s" s="2">
         <v>76</v>
       </c>
@@ -1929,7 +2009,7 @@
         <v>76</v>
       </c>
       <c r="S10" t="s" s="2">
-        <v>76</v>
+        <v>140</v>
       </c>
       <c r="T10" t="s" s="2">
         <v>76</v>
@@ -1968,13 +2048,13 @@
         <v>76</v>
       </c>
       <c r="AF10" t="s" s="2">
-        <v>152</v>
+        <v>135</v>
       </c>
       <c r="AG10" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH10" t="s" s="2">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="AI10" t="s" s="2">
         <v>76</v>
@@ -1983,17 +2063,689 @@
         <v>83</v>
       </c>
       <c r="AK10" t="s" s="2">
+        <v>136</v>
+      </c>
+      <c r="AL10" t="s" s="2">
+        <v>137</v>
+      </c>
+      <c r="AM10" t="s" s="2">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="11" hidden="true">
+      <c r="A11" t="s" s="2">
+        <v>141</v>
+      </c>
+      <c r="B11" t="s" s="2">
+        <v>128</v>
+      </c>
+      <c r="C11" t="s" s="2">
+        <v>142</v>
+      </c>
+      <c r="D11" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="E11" s="2"/>
+      <c r="F11" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="G11" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="H11" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="I11" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="J11" t="s" s="2">
+        <v>105</v>
+      </c>
+      <c r="K11" t="s" s="2">
+        <v>129</v>
+      </c>
+      <c r="L11" t="s" s="2">
+        <v>130</v>
+      </c>
+      <c r="M11" t="s" s="2">
+        <v>131</v>
+      </c>
+      <c r="N11" t="s" s="2">
+        <v>132</v>
+      </c>
+      <c r="O11" t="s" s="2">
+        <v>133</v>
+      </c>
+      <c r="P11" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Q11" s="2"/>
+      <c r="R11" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="S11" t="s" s="2">
+        <v>143</v>
+      </c>
+      <c r="T11" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="U11" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="V11" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="W11" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="X11" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Y11" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Z11" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AA11" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AB11" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AC11" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AD11" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AE11" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AF11" t="s" s="2">
+        <v>135</v>
+      </c>
+      <c r="AG11" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AH11" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AI11" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AJ11" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AK11" t="s" s="2">
+        <v>136</v>
+      </c>
+      <c r="AL11" t="s" s="2">
+        <v>137</v>
+      </c>
+      <c r="AM11" t="s" s="2">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="12" hidden="true">
+      <c r="A12" t="s" s="2">
+        <v>144</v>
+      </c>
+      <c r="B12" t="s" s="2">
+        <v>144</v>
+      </c>
+      <c r="C12" s="2"/>
+      <c r="D12" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="E12" s="2"/>
+      <c r="F12" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="G12" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="H12" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="I12" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="J12" t="s" s="2">
+        <v>105</v>
+      </c>
+      <c r="K12" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="L12" t="s" s="2">
+        <v>145</v>
+      </c>
+      <c r="M12" t="s" s="2">
+        <v>146</v>
+      </c>
+      <c r="N12" t="s" s="2">
+        <v>147</v>
+      </c>
+      <c r="O12" t="s" s="2">
+        <v>148</v>
+      </c>
+      <c r="P12" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Q12" s="2"/>
+      <c r="R12" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="S12" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="T12" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="U12" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="V12" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="W12" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="X12" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Y12" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Z12" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AA12" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AB12" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AC12" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AD12" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AE12" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AF12" t="s" s="2">
+        <v>149</v>
+      </c>
+      <c r="AG12" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AH12" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="AI12" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AJ12" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AK12" t="s" s="2">
+        <v>150</v>
+      </c>
+      <c r="AL12" t="s" s="2">
+        <v>151</v>
+      </c>
+      <c r="AM12" t="s" s="2">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s" s="2">
+        <v>152</v>
+      </c>
+      <c r="B13" t="s" s="2">
+        <v>152</v>
+      </c>
+      <c r="C13" s="2"/>
+      <c r="D13" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="E13" s="2"/>
+      <c r="F13" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="G13" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="H13" t="s" s="2">
+        <v>105</v>
+      </c>
+      <c r="I13" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="J13" t="s" s="2">
+        <v>105</v>
+      </c>
+      <c r="K13" t="s" s="2">
+        <v>153</v>
+      </c>
+      <c r="L13" t="s" s="2">
+        <v>154</v>
+      </c>
+      <c r="M13" t="s" s="2">
+        <v>155</v>
+      </c>
+      <c r="N13" t="s" s="2">
+        <v>156</v>
+      </c>
+      <c r="O13" t="s" s="2">
         <v>157</v>
       </c>
-      <c r="AL10" t="s" s="2">
+      <c r="P13" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Q13" s="2"/>
+      <c r="R13" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="S13" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="T13" t="s" s="2">
         <v>158</v>
       </c>
-      <c r="AM10" t="s" s="2">
+      <c r="U13" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="V13" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="W13" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="X13" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Y13" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Z13" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AA13" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AB13" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AC13" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AD13" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AE13" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AF13" t="s" s="2">
+        <v>152</v>
+      </c>
+      <c r="AG13" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AH13" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="AI13" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AJ13" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AK13" t="s" s="2">
         <v>159</v>
       </c>
+      <c r="AL13" t="s" s="2">
+        <v>160</v>
+      </c>
+      <c r="AM13" t="s" s="2">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s" s="2">
+        <v>162</v>
+      </c>
+      <c r="B14" t="s" s="2">
+        <v>162</v>
+      </c>
+      <c r="C14" s="2"/>
+      <c r="D14" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="E14" s="2"/>
+      <c r="F14" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="G14" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="H14" t="s" s="2">
+        <v>105</v>
+      </c>
+      <c r="I14" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="J14" t="s" s="2">
+        <v>105</v>
+      </c>
+      <c r="K14" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="L14" t="s" s="2">
+        <v>163</v>
+      </c>
+      <c r="M14" t="s" s="2">
+        <v>164</v>
+      </c>
+      <c r="N14" t="s" s="2">
+        <v>165</v>
+      </c>
+      <c r="O14" s="2"/>
+      <c r="P14" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Q14" s="2"/>
+      <c r="R14" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="S14" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="T14" t="s" s="2">
+        <v>166</v>
+      </c>
+      <c r="U14" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="V14" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="W14" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="X14" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Y14" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Z14" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AA14" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AB14" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AC14" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AD14" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AE14" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AF14" t="s" s="2">
+        <v>162</v>
+      </c>
+      <c r="AG14" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AH14" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="AI14" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AJ14" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AK14" t="s" s="2">
+        <v>167</v>
+      </c>
+      <c r="AL14" t="s" s="2">
+        <v>168</v>
+      </c>
+      <c r="AM14" t="s" s="2">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="15" hidden="true">
+      <c r="A15" t="s" s="2">
+        <v>170</v>
+      </c>
+      <c r="B15" t="s" s="2">
+        <v>170</v>
+      </c>
+      <c r="C15" s="2"/>
+      <c r="D15" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="E15" s="2"/>
+      <c r="F15" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="G15" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="H15" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="I15" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="J15" t="s" s="2">
+        <v>105</v>
+      </c>
+      <c r="K15" t="s" s="2">
+        <v>171</v>
+      </c>
+      <c r="L15" t="s" s="2">
+        <v>172</v>
+      </c>
+      <c r="M15" t="s" s="2">
+        <v>173</v>
+      </c>
+      <c r="N15" s="2"/>
+      <c r="O15" s="2"/>
+      <c r="P15" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Q15" s="2"/>
+      <c r="R15" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="S15" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="T15" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="U15" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="V15" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="W15" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="X15" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Y15" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Z15" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AA15" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AB15" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AC15" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AD15" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AE15" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AF15" t="s" s="2">
+        <v>170</v>
+      </c>
+      <c r="AG15" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AH15" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="AI15" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AJ15" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AK15" t="s" s="2">
+        <v>174</v>
+      </c>
+      <c r="AL15" t="s" s="2">
+        <v>175</v>
+      </c>
+      <c r="AM15" t="s" s="2">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="16" hidden="true">
+      <c r="A16" t="s" s="2">
+        <v>177</v>
+      </c>
+      <c r="B16" t="s" s="2">
+        <v>177</v>
+      </c>
+      <c r="C16" s="2"/>
+      <c r="D16" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="E16" s="2"/>
+      <c r="F16" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="G16" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="H16" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="I16" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="J16" t="s" s="2">
+        <v>105</v>
+      </c>
+      <c r="K16" t="s" s="2">
+        <v>178</v>
+      </c>
+      <c r="L16" t="s" s="2">
+        <v>179</v>
+      </c>
+      <c r="M16" t="s" s="2">
+        <v>180</v>
+      </c>
+      <c r="N16" t="s" s="2">
+        <v>181</v>
+      </c>
+      <c r="O16" s="2"/>
+      <c r="P16" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Q16" s="2"/>
+      <c r="R16" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="S16" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="T16" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="U16" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="V16" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="W16" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="X16" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Y16" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Z16" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AA16" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AB16" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AC16" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AD16" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AE16" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AF16" t="s" s="2">
+        <v>177</v>
+      </c>
+      <c r="AG16" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AH16" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="AI16" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AJ16" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AK16" t="s" s="2">
+        <v>182</v>
+      </c>
+      <c r="AL16" t="s" s="2">
+        <v>183</v>
+      </c>
+      <c r="AM16" t="s" s="2">
+        <v>184</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AM10">
+  <autoFilter ref="A1:AM16">
     <filterColumn colId="7">
       <customFilters>
         <customFilter operator="notEqual" val=" "/>
@@ -2003,7 +2755,7 @@
       <filters blank="true"/>
     </filterColumn>
   </autoFilter>
-  <conditionalFormatting sqref="A2:AI9">
+  <conditionalFormatting sqref="A2:AI15">
     <cfRule type="expression" dxfId="0" priority="1">
       <formula>$G2&lt;&gt;"Y"</formula>
     </cfRule>

</xml_diff>